<commit_message>
Shift case study to the 2026-27 financial year
The baseline ran Apr-2025 to Mar-2026 with a data date of Sep-2025,
which put the project's "current" reporting position a year in the past
at submission. Now Apr-2026 to Mar-2027 with a data date of Sep-2026, so
the case reads as a live project one month behind the reporting date.

Numerically identical - only the period labels changed. Benchmark
rebuilt and revalidated: 50 of 50 comparisons still agree. Dashboard
screenshots retaken.
</commit_message>
<xml_diff>
--- a/benchmark/EVM_Manual_Benchmark.xlsx
+++ b/benchmark/EVM_Manual_Benchmark.xlsx
@@ -560,7 +560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Data date    end of Period 6 (Sep-2025)</t>
+          <t>Data date    end of Period 6 (Sep-2026)</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Earned Value by Work Package — end of Period 5 (Aug-2025)</t>
+          <t>Earned Value by Work Package — end of Period 5 (Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Earned Value by Work Package — end of Period 6 (Sep-2025)</t>
+          <t>Earned Value by Work Package — end of Period 6 (Sep-2026)</t>
         </is>
       </c>
     </row>

</xml_diff>